<commit_message>
feat: trade Zeeshan Ansari out for T Natarajan in SRH roster
</commit_message>
<xml_diff>
--- a/data/squadofsunrisers.xlsx
+++ b/data/squadofsunrisers.xlsx
@@ -572,7 +572,6 @@
           <t>England</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -595,7 +594,6 @@
           <t>England</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -645,7 +643,6 @@
           <t>England</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -668,7 +665,6 @@
           <t>England</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -691,7 +687,6 @@
           <t>England</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -768,7 +763,6 @@
           <t>England</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -791,7 +785,6 @@
           <t>England</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -814,7 +807,6 @@
           <t>England</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1026,7 +1018,6 @@
           <t>England</t>
         </is>
       </c>
-      <c r="E24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1211,7 +1202,6 @@
           <t>England</t>
         </is>
       </c>
-      <c r="E31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -1288,7 +1278,6 @@
           <t>England</t>
         </is>
       </c>
-      <c r="E34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -1311,7 +1300,6 @@
           <t>England</t>
         </is>
       </c>
-      <c r="E35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -1415,7 +1403,6 @@
           <t>England</t>
         </is>
       </c>
-      <c r="E39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -1438,7 +1425,6 @@
           <t>England</t>
         </is>
       </c>
-      <c r="E40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -1542,7 +1528,6 @@
           <t>India</t>
         </is>
       </c>
-      <c r="E44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -1646,7 +1631,6 @@
           <t>India</t>
         </is>
       </c>
-      <c r="E48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -1669,7 +1653,6 @@
           <t>India</t>
         </is>
       </c>
-      <c r="E49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -1692,7 +1675,6 @@
           <t>India</t>
         </is>
       </c>
-      <c r="E50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -1715,7 +1697,6 @@
           <t>India</t>
         </is>
       </c>
-      <c r="E51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -1738,7 +1719,6 @@
           <t>India</t>
         </is>
       </c>
-      <c r="E52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -1788,7 +1768,6 @@
           <t>India</t>
         </is>
       </c>
-      <c r="E54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -1811,7 +1790,6 @@
           <t>India</t>
         </is>
       </c>
-      <c r="E55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -1834,7 +1812,6 @@
           <t>India</t>
         </is>
       </c>
-      <c r="E56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -1871,7 +1848,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Zeeshan Ansari</t>
+          <t>T Natarajan</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
@@ -1884,7 +1861,6 @@
           <t>India</t>
         </is>
       </c>
-      <c r="E58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -1907,7 +1883,6 @@
           <t>India</t>
         </is>
       </c>
-      <c r="E59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -1930,7 +1905,6 @@
           <t>India</t>
         </is>
       </c>
-      <c r="E60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -1953,7 +1927,6 @@
           <t>India</t>
         </is>
       </c>
-      <c r="E61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -1976,7 +1949,6 @@
           <t>India</t>
         </is>
       </c>
-      <c r="E62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -1999,7 +1971,6 @@
           <t>India</t>
         </is>
       </c>
-      <c r="E63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -2292,7 +2263,6 @@
           <t>South Africa</t>
         </is>
       </c>
-      <c r="E74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -2342,7 +2312,6 @@
           <t>South Africa</t>
         </is>
       </c>
-      <c r="E76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -2365,7 +2334,6 @@
           <t>South Africa</t>
         </is>
       </c>
-      <c r="E77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -2442,7 +2410,6 @@
           <t>South Africa</t>
         </is>
       </c>
-      <c r="E80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -2492,7 +2459,6 @@
           <t>South Africa</t>
         </is>
       </c>
-      <c r="E82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -2542,7 +2508,6 @@
           <t>South Africa</t>
         </is>
       </c>
-      <c r="E84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -2565,7 +2530,6 @@
           <t>South Africa</t>
         </is>
       </c>
-      <c r="E85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -2588,7 +2552,6 @@
           <t>South Africa</t>
         </is>
       </c>
-      <c r="E86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -2611,7 +2574,6 @@
           <t>South Africa</t>
         </is>
       </c>
-      <c r="E87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -2634,7 +2596,6 @@
           <t>South Africa</t>
         </is>
       </c>
-      <c r="E88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -2684,7 +2645,6 @@
           <t>South Africa</t>
         </is>
       </c>
-      <c r="E90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">

</xml_diff>